<commit_message>
found data, added data onto xlsx file for hurricane melissa, there are some gaps though
</commit_message>
<xml_diff>
--- a/week5/data/Databases-week5-task.xlsx
+++ b/week5/data/Databases-week5-task.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/My-Disk/Uni/databases/week3/createSchema/Databases-Group17-hurricanesDB/week5/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B49F8EEE-33E2-6544-B8B3-5088FCAF5322}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADD39C86-F6FD-5548-AEC7-4A64A44FD2F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21460" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="205">
   <si>
     <t>Hurricane Impact Database — ERD Overview</t>
   </si>
@@ -362,6 +362,303 @@
   </si>
   <si>
     <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Haiti: at least 43 deaths, 25 in Petit-Goave (PDF p.12 table; p.13); cause breakdown not known so direct/indirect left blank. No USD damage estimate given.</t>
+  </si>
+  <si>
+    <t>New Hope Primary School, Westmoreland Parish</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.27 (station, coordinates, sustained 47 kt, gust 114 kt at 1600 UTC 28 Oct, min pressure 913.5 mb). Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>Hampden, Trelawny Parish</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.27 (sustained 57 kt, gust 105 kt, min pressure 958 mb). Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>Bamboo, St. Ann Parish</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.26 (sustained 45 kt, gust 90 kt, min pressure 972.5 mb). Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>Appleton Estate, St. Elizabeth Parish</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.26 (sustained 40 kt, gust 96 kt, min pressure 964.6 mb). Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>Mountainside Primary School, Westmoreland Parish</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.27 (sustained 56 kt, gust 90 kt, min pressure 974.8 mb, rain 20.01 in). Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>Newcombe Valley Primary School, Westmoreland Parish</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.27 (sustained 54 kt, gust 93 kt, min pressure 972.5 mb). Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>Orange Valley, Trelawny Parish</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.27 (sustained 44 kt, gust 88 kt, min pressure 960.2 mb, rain 9.29 in). Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>Minards, St. Ann Parish</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.26 (sustained 44 kt, gust 85 kt, min pressure 965.9 mb, rain 10.66 in). Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>Mason River, Clarendon Parish</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.24 (sustained 25 kt, gust 68 kt, min pressure 984.1 mb, rain 13.16 in). Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>Woodford, Kingston &amp; St. Andrew Parish</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.25 (sustained 37 kt, gust 69 kt, min pressure 993.7 mb, rain 7.35 in). Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>Mavis Bank, Kingston &amp; St. Andrew Parish</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.25 (sustained 10 kt, gust 37 kt, min pressure 993.6 mb, rain 22.32 in). Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>Sangster International Airport, Montego Bay (MKJS)</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.24 (ICAO site; sustained 40 kt, gust 56 kt, min pressure 998.0 mb; no data after 1000 UTC 28 Oct). Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>Norman Manley International Airport, Kingston (MKJP)</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.24 (ICAO site; sustained 41 kt, gust 50 kt, min pressure 995.9 mb). Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>Contramaestre (78363), Santiago de Cuba Province</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.28 (INSMET station; sustained 59 kt (10-min), gust 101 kt, min pressure 967.7 mb, rain 14.71 in); eye passed over 0845–0856 UTC 29 Oct (text p.8). Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>Gran Piedra (78366), Santiago de Cuba Province</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.28 (INSMET elevated station; sustained 70 kt (10-min), gust 118 kt, rain 13.20 in); highest sustained wind and gust in Cuba (text p.8). Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>Leeward Point Field, Guantanamo Bay (MUGM)</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.28 (ICAO site; sustained 51 kt, gust 65 kt, min pressure 996.5 mb, rain 6.50 in; data gap 0751–2151 UTC 29 Oct). Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>Guaro (78370), Holguin Province</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.29 (INSMET station; sustained 62 kt (10-min), gust 68 kt, min pressure 983.4 mb, rain 10.84 in). Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>Jucarito (78361), Granma Province</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.29 (INSMET station; sustained 47 kt (10-min), gust 68 kt, min pressure 999.0 mb, rain 4.04 in). Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>Sea Horse Shores #83, Pitts Town, Crooked Island</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.32 (sustained 66 kt, gust 77 kt, min pressure 980.7 mb); strongest winds recorded in the Bahamas (text p.8). Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>Indian Hole Point, Long Island</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.32 (sustained 45 kt, gust 61 kt, min pressure 968.8 mb). Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>Buckley's Settlement, Long Island</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.32 (sustained 35 kt, gust 44 kt, min pressure 966.5 mb; Weather Underground site with ~6 mb low bias, text p.8). Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>Cockburn Town, San Salvador Island</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.32 and text p.11: highest Bahamas rainfall 7.78 in / 198 mm. Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>L.F. Wade International Airport (TXKF)</t>
+  </si>
+  <si>
+    <t>Bermuda</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.29 (ICAO site; sustained 43 kt, gust 60 kt, min pressure 996.9 mb). Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>National Museum of Bermuda (NMB)</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.29 (sustained 68 kt at 46 m elevation, gust 86 kt, min pressure 991.9 mb). Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>Saint Louis du Sud, Sud Department</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Text p.10 (35.16 in / 893 mm, second-highest total in Haiti); Table 3, PDF p.30. Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>Annette, Grand'Anse Department</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Text p.10 (33.72 in / 856.5 mm); Table 3, PDF p.30. Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>Vieux Bourg d'Aquin, Sud Department</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Text p.10 (32.90 in / 835.6 mm); Table 3, PDF p.30. Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>Polo, Barahona Province (highest rainfall in Dominican Republic)</t>
+  </si>
+  <si>
+    <t>Dominican Republic</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Text p.11 (29.02 in / 737.2 mm); Table 3, PDF p.31. Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>Centro de los Heroes (EMA), Distrito Nacional (Santo Domingo)</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Text p.11 (19.98 in / 507.4 mm); Table 3, PDF p.31. Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>Santo Domingo Este, Santo Domingo Province</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Text p.11 (17.84 in / 453.1 mm); Table 3, PDF p.31. Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>Panama (country level)</t>
+  </si>
+  <si>
+    <t>Panama</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Casualty table PDF p.12 and text p.15: moisture associated with Melissa caused heavy rain and flooding that contributed to three fatalities. Longitude negative = °W.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.27 (station, coordinates, sustained 47 kt, gust 114 kt at 1600 UTC 28 Oct, min pressure 913.5 mb). Site of the highest gust reported in Jamaica (text p.6–7). Jamaica station sustained wind = 1-hour average (Table 3 footnote b, PDF p.32). No rainfall reported. Window = time of reported maximum sustained wind. avg_wind_speed (kt) = reported sustained wind at the station, not a best-track average. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.27 (sustained 57 kt, gust 105 kt, min pressure 958 mb). Jamaica station sustained wind = 1-hour average (Table 3 footnote b, PDF p.32). No rainfall reported. Window = time of reported maximum sustained wind. avg_wind_speed (kt) = reported sustained wind at the station, not a best-track average. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.26 (sustained 45 kt, gust 90 kt, min pressure 972.5 mb). Jamaica station sustained wind = 1-hour average (Table 3 footnote b, PDF p.32). Table rainfall (4.43 in) is flagged with an unexplained asterisk, so left blank. Window = time of reported maximum sustained wind. avg_wind_speed (kt) = reported sustained wind at the station, not a best-track average. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.26 (sustained 40 kt, gust 96 kt, min pressure 964.6 mb). Jamaica station sustained wind = 1-hour average (Table 3 footnote b, PDF p.32). No rainfall reported. Window = time of reported maximum sustained wind. avg_wind_speed (kt) = reported sustained wind at the station, not a best-track average. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.27 (sustained 56 kt, gust 90 kt, min pressure 974.8 mb, rain 20.01 in). Jamaica station sustained wind = 1-hour average (Table 3 footnote b, PDF p.32). Rainfall converted from inches (x25.4). Window = time of reported maximum sustained wind. avg_wind_speed (kt) = reported sustained wind at the station, not a best-track average. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.27 (sustained 54 kt, gust 93 kt, min pressure 972.5 mb). Jamaica station sustained wind = 1-hour average (Table 3 footnote b, PDF p.32). No rainfall reported. Window = time of reported maximum sustained wind. avg_wind_speed (kt) = reported sustained wind at the station, not a best-track average. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.27 (sustained 44 kt, gust 88 kt, min pressure 960.2 mb, rain 9.29 in). Jamaica station sustained wind = 1-hour average (Table 3 footnote b, PDF p.32). Rainfall converted from inches (x25.4). Window = time of reported maximum sustained wind. avg_wind_speed (kt) = reported sustained wind at the station, not a best-track average. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.26 (sustained 44 kt, gust 85 kt, min pressure 965.9 mb, rain 10.66 in). Jamaica station sustained wind = 1-hour average (Table 3 footnote b, PDF p.32). Rainfall converted from inches (x25.4). Window = time of reported maximum sustained wind. avg_wind_speed (kt) = reported sustained wind at the station, not a best-track average. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.24 (sustained 25 kt, gust 68 kt, min pressure 984.1 mb, rain 13.16 in). Jamaica station sustained wind = 1-hour average (Table 3 footnote b, PDF p.32). Rainfall converted from inches (x25.4). Window = time of reported maximum sustained wind. avg_wind_speed (kt) = reported sustained wind at the station, not a best-track average. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.25 (sustained 37 kt, gust 69 kt, min pressure 993.7 mb, rain 7.35 in). Strongest gust in the Kingston area (text p.7). Jamaica station sustained wind = 1-hour average (Table 3 footnote b, PDF p.32). Rainfall converted from inches (x25.4). Window = time of reported maximum sustained wind. avg_wind_speed (kt) = reported sustained wind at the station, not a best-track average. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.25 (sustained 10 kt, gust 37 kt, min pressure 993.6 mb, rain 22.32 in). Jamaica station sustained wind = 1-hour average (Table 3 footnote b, PDF p.32). Rainfall converted from inches (x25.4). Window = time of reported maximum sustained wind. avg_wind_speed (kt) = reported sustained wind at the station, not a best-track average. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.24 (ICAO site; sustained 40 kt, gust 56 kt, min pressure 998.0 mb; no data after 1000 UTC 28 Oct). ICAO sustained wind = 2-min average (footnote b, p.32). No rainfall reported. Window = time of reported maximum sustained wind. avg_wind_speed (kt) = reported sustained wind at the station, not a best-track average. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.24 (ICAO site; sustained 41 kt, gust 50 kt, min pressure 995.9 mb). ICAO sustained wind = 2-min average (footnote b, p.32). No rainfall reported. Window = time of reported maximum sustained wind. avg_wind_speed (kt) = reported sustained wind at the station, not a best-track average. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.28 (INSMET station; sustained 59 kt (10-min), gust 101 kt, min pressure 967.7 mb, rain 14.71 in); eye passed over 0845–0856 UTC 29 Oct (text p.8). Report gives no coordinates. Rainfall converted from inches (x25.4). Window = time of reported maximum sustained wind. avg_wind_speed (kt) = reported sustained wind at the station, not a best-track average. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.28 (INSMET elevated station; sustained 70 kt (10-min), gust 118 kt, rain 13.20 in); highest sustained wind and gust in Cuba (text p.8). Report gives no coordinates. Rainfall converted from inches (x25.4). Window = time of reported maximum sustained wind. avg_wind_speed (kt) = reported sustained wind at the station, not a best-track average. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.28 (ICAO site; sustained 51 kt, gust 65 kt, min pressure 996.5 mb, rain 6.50 in; data gap 0751–2151 UTC 29 Oct). Coordinates printed in the table duplicate those of the Santiago airport, so left blank. Rainfall converted from inches (x25.4). Window = time of reported maximum sustained wind. avg_wind_speed (kt) = reported sustained wind at the station, not a best-track average. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.29 (INSMET station; sustained 62 kt (10-min), gust 68 kt, min pressure 983.4 mb, rain 10.84 in). Report gives no coordinates. Rainfall converted from inches (x25.4). Window = time of reported maximum sustained wind. avg_wind_speed (kt) = reported sustained wind at the station, not a best-track average. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.29 (INSMET station; sustained 47 kt (10-min), gust 68 kt, min pressure 999.0 mb, rain 4.04 in). Report gives no coordinates. Rainfall converted from inches (x25.4). Window = time of reported maximum sustained wind. avg_wind_speed (kt) = reported sustained wind at the station, not a best-track average. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.32 (sustained 66 kt, gust 77 kt, min pressure 980.7 mb); strongest winds recorded in the Bahamas (text p.8). No rainfall reported. Window = time of reported maximum sustained wind. avg_wind_speed (kt) = reported sustained wind at the station, not a best-track average. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.32 (sustained 45 kt, gust 61 kt, min pressure 968.8 mb). No rainfall reported. Window = time of reported maximum sustained wind. avg_wind_speed (kt) = reported sustained wind at the station, not a best-track average. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.32 (sustained 35 kt, gust 44 kt, min pressure 966.5 mb; Weather Underground site with ~6 mb low bias, text p.8). No rainfall reported. Window = time of reported maximum sustained wind. avg_wind_speed (kt) = reported sustained wind at the station, not a best-track average. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.32 and text p.11: highest Bahamas rainfall 7.78 in / 198 mm. No wind reported at this site. Observation window not specified in the report. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.29 (ICAO site; sustained 43 kt, gust 60 kt, min pressure 996.9 mb). Impacts minor, no casualties (text p.15). No rainfall reported. Window = time of reported maximum sustained wind. avg_wind_speed (kt) = reported sustained wind at the station, not a best-track average. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Table 3, PDF p.29 (sustained 68 kt at 46 m elevation, gust 86 kt, min pressure 991.9 mb). No rainfall reported. Window = time of reported maximum sustained wind. avg_wind_speed (kt) = reported sustained wind at the station, not a best-track average. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Text p.10 (35.16 in / 893 mm, second-highest total in Haiti); Table 3, PDF p.30. Report gives no coordinates or wind data. Observation window not specified in the report. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Text p.10 (33.72 in / 856.5 mm); Table 3, PDF p.30. Report gives no coordinates or wind data. Observation window not specified in the report. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Text p.10 (32.90 in / 835.6 mm); Table 3, PDF p.30. Report gives no coordinates or wind data. Observation window not specified in the report. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Text p.11 (29.02 in / 737.2 mm); Table 3, PDF p.31. Report gives no coordinates or wind data. Observation window not specified in the report. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Text p.11 (19.98 in / 507.4 mm); Table 3, PDF p.31. Report gives no coordinates or wind data. Observation window not specified in the report. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Text p.11 (17.84 in / 453.1 mm); Table 3, PDF p.31. Report gives no coordinates or wind data. Observation window not specified in the report. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Casualty table PDF p.12 and text p.15: moisture associated with Melissa caused heavy rain and flooding that contributed to three fatalities. No stations, coordinates, wind or rainfall reported. Observation window not specified in the report. avg_temperature: not reported.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Panama: heavy rain and flooding contributed to three fatalities (PDF p.15; total in casualty table p.12). Direct/indirect split not reported, so left blank. No USD damage given.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Bermuda: impacts minor; 'no reported casualties' (PDF p.15), recorded as 0 direct / 0 indirect. No USD damage given.</t>
+  </si>
+  <si>
+    <t>NHC Tropical Cyclone Report: Hurricane Melissa (AL132025), 19 May 2026 revised version, https://www.nhc.noaa.gov/data/tcr/AL132025_Melissa.pdf — Dominican Republic: government assessment reported no fatalities attributed to Melissa (PDF p.14), recorded as 0. Damage reported as counts only (823 homes flooded, 21 partially affected, 2 destroyed, 29 aqueducts out of service affecting ~250,000 users; p.14), no USD figure.</t>
   </si>
 </sst>
 </file>
@@ -374,7 +671,7 @@
     <numFmt numFmtId="166" formatCode="0.0"/>
     <numFmt numFmtId="168" formatCode="[$$-409]#,##0"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -461,6 +758,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -521,7 +825,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -576,6 +880,21 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="168" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -6337,7 +6656,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D02AE60-BF3F-44DB-B63B-ADBA2211271F}">
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.1640625" customWidth="1"/>
@@ -6533,6 +6852,780 @@
         <v>102</v>
       </c>
     </row>
+    <row r="10" spans="1:9" ht="112" x14ac:dyDescent="0.2">
+      <c r="A10" s="30">
+        <v>4</v>
+      </c>
+      <c r="B10" s="30">
+        <v>0</v>
+      </c>
+      <c r="C10" s="30">
+        <v>4</v>
+      </c>
+      <c r="D10" s="32">
+        <v>45958.666666666664</v>
+      </c>
+      <c r="E10" s="32">
+        <v>45958.666666666664</v>
+      </c>
+      <c r="F10" s="30">
+        <v>47</v>
+      </c>
+      <c r="G10" s="33"/>
+      <c r="H10" s="30"/>
+      <c r="I10" s="31" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="96" x14ac:dyDescent="0.2">
+      <c r="A11" s="30">
+        <v>5</v>
+      </c>
+      <c r="B11" s="30">
+        <v>0</v>
+      </c>
+      <c r="C11" s="30">
+        <v>5</v>
+      </c>
+      <c r="D11" s="32">
+        <v>45958.833333333336</v>
+      </c>
+      <c r="E11" s="32">
+        <v>45958.833333333336</v>
+      </c>
+      <c r="F11" s="30">
+        <v>57</v>
+      </c>
+      <c r="G11" s="33"/>
+      <c r="H11" s="30"/>
+      <c r="I11" s="31" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="112" x14ac:dyDescent="0.2">
+      <c r="A12" s="30">
+        <v>6</v>
+      </c>
+      <c r="B12" s="30">
+        <v>0</v>
+      </c>
+      <c r="C12" s="30">
+        <v>6</v>
+      </c>
+      <c r="D12" s="32">
+        <v>45958.958333333336</v>
+      </c>
+      <c r="E12" s="32">
+        <v>45958.958333333336</v>
+      </c>
+      <c r="F12" s="30">
+        <v>45</v>
+      </c>
+      <c r="G12" s="33"/>
+      <c r="H12" s="30"/>
+      <c r="I12" s="31" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="96" x14ac:dyDescent="0.2">
+      <c r="A13" s="30">
+        <v>7</v>
+      </c>
+      <c r="B13" s="30">
+        <v>0</v>
+      </c>
+      <c r="C13" s="30">
+        <v>7</v>
+      </c>
+      <c r="D13" s="32">
+        <v>45958.75</v>
+      </c>
+      <c r="E13" s="32">
+        <v>45958.75</v>
+      </c>
+      <c r="F13" s="30">
+        <v>40</v>
+      </c>
+      <c r="G13" s="33"/>
+      <c r="H13" s="30"/>
+      <c r="I13" s="31" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="112" x14ac:dyDescent="0.2">
+      <c r="A14" s="30">
+        <v>8</v>
+      </c>
+      <c r="B14" s="30">
+        <v>0</v>
+      </c>
+      <c r="C14" s="30">
+        <v>8</v>
+      </c>
+      <c r="D14" s="32">
+        <v>45958.708333333336</v>
+      </c>
+      <c r="E14" s="32">
+        <v>45958.708333333336</v>
+      </c>
+      <c r="F14" s="30">
+        <v>56</v>
+      </c>
+      <c r="G14" s="33">
+        <f>ROUND(20.01*25.4,1)</f>
+        <v>508.3</v>
+      </c>
+      <c r="H14" s="30"/>
+      <c r="I14" s="31" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="96" x14ac:dyDescent="0.2">
+      <c r="A15" s="30">
+        <v>9</v>
+      </c>
+      <c r="B15" s="30">
+        <v>0</v>
+      </c>
+      <c r="C15" s="30">
+        <v>9</v>
+      </c>
+      <c r="D15" s="32">
+        <v>45958.625</v>
+      </c>
+      <c r="E15" s="32">
+        <v>45958.625</v>
+      </c>
+      <c r="F15" s="30">
+        <v>54</v>
+      </c>
+      <c r="G15" s="33"/>
+      <c r="H15" s="30"/>
+      <c r="I15" s="31" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="112" x14ac:dyDescent="0.2">
+      <c r="A16" s="30">
+        <v>10</v>
+      </c>
+      <c r="B16" s="30">
+        <v>0</v>
+      </c>
+      <c r="C16" s="30">
+        <v>10</v>
+      </c>
+      <c r="D16" s="32">
+        <v>45958.833333333336</v>
+      </c>
+      <c r="E16" s="32">
+        <v>45958.833333333336</v>
+      </c>
+      <c r="F16" s="30">
+        <v>44</v>
+      </c>
+      <c r="G16" s="33">
+        <f>ROUND(9.29*25.4,1)</f>
+        <v>236</v>
+      </c>
+      <c r="H16" s="30"/>
+      <c r="I16" s="31" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="112" x14ac:dyDescent="0.2">
+      <c r="A17" s="30">
+        <v>11</v>
+      </c>
+      <c r="B17" s="30">
+        <v>0</v>
+      </c>
+      <c r="C17" s="30">
+        <v>11</v>
+      </c>
+      <c r="D17" s="32">
+        <v>45958.916666666664</v>
+      </c>
+      <c r="E17" s="32">
+        <v>45958.916666666664</v>
+      </c>
+      <c r="F17" s="30">
+        <v>44</v>
+      </c>
+      <c r="G17" s="33">
+        <f>ROUND(10.66*25.4,1)</f>
+        <v>270.8</v>
+      </c>
+      <c r="H17" s="30"/>
+      <c r="I17" s="31" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="112" x14ac:dyDescent="0.2">
+      <c r="A18" s="30">
+        <v>12</v>
+      </c>
+      <c r="B18" s="30">
+        <v>0</v>
+      </c>
+      <c r="C18" s="30">
+        <v>12</v>
+      </c>
+      <c r="D18" s="32">
+        <v>45958.833333333336</v>
+      </c>
+      <c r="E18" s="32">
+        <v>45958.833333333336</v>
+      </c>
+      <c r="F18" s="30">
+        <v>25</v>
+      </c>
+      <c r="G18" s="33">
+        <f>ROUND(13.16*25.4,1)</f>
+        <v>334.3</v>
+      </c>
+      <c r="H18" s="30"/>
+      <c r="I18" s="31" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="112" x14ac:dyDescent="0.2">
+      <c r="A19" s="30">
+        <v>13</v>
+      </c>
+      <c r="B19" s="30">
+        <v>0</v>
+      </c>
+      <c r="C19" s="30">
+        <v>13</v>
+      </c>
+      <c r="D19" s="32">
+        <v>45958.75</v>
+      </c>
+      <c r="E19" s="32">
+        <v>45958.75</v>
+      </c>
+      <c r="F19" s="30">
+        <v>37</v>
+      </c>
+      <c r="G19" s="33">
+        <f>ROUND(7.35*25.4,1)</f>
+        <v>186.7</v>
+      </c>
+      <c r="H19" s="30"/>
+      <c r="I19" s="31" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="112" x14ac:dyDescent="0.2">
+      <c r="A20" s="30">
+        <v>14</v>
+      </c>
+      <c r="B20" s="30">
+        <v>0</v>
+      </c>
+      <c r="C20" s="30">
+        <v>14</v>
+      </c>
+      <c r="D20" s="32">
+        <v>45958.583333333336</v>
+      </c>
+      <c r="E20" s="32">
+        <v>45958.583333333336</v>
+      </c>
+      <c r="F20" s="30">
+        <v>10</v>
+      </c>
+      <c r="G20" s="33">
+        <f>ROUND(22.32*25.4,1)</f>
+        <v>566.9</v>
+      </c>
+      <c r="H20" s="30"/>
+      <c r="I20" s="31" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="96" x14ac:dyDescent="0.2">
+      <c r="A21" s="30">
+        <v>15</v>
+      </c>
+      <c r="B21" s="30">
+        <v>0</v>
+      </c>
+      <c r="C21" s="30">
+        <v>15</v>
+      </c>
+      <c r="D21" s="32">
+        <v>45958.333333333336</v>
+      </c>
+      <c r="E21" s="32">
+        <v>45958.333333333336</v>
+      </c>
+      <c r="F21" s="30">
+        <v>40</v>
+      </c>
+      <c r="G21" s="33"/>
+      <c r="H21" s="30"/>
+      <c r="I21" s="31" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="96" x14ac:dyDescent="0.2">
+      <c r="A22" s="30">
+        <v>16</v>
+      </c>
+      <c r="B22" s="30">
+        <v>0</v>
+      </c>
+      <c r="C22" s="30">
+        <v>16</v>
+      </c>
+      <c r="D22" s="32">
+        <v>45958.791666666664</v>
+      </c>
+      <c r="E22" s="32">
+        <v>45958.791666666664</v>
+      </c>
+      <c r="F22" s="30">
+        <v>41</v>
+      </c>
+      <c r="G22" s="33"/>
+      <c r="H22" s="30"/>
+      <c r="I22" s="31" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="112" x14ac:dyDescent="0.2">
+      <c r="A23" s="30">
+        <v>17</v>
+      </c>
+      <c r="B23" s="30">
+        <v>0</v>
+      </c>
+      <c r="C23" s="30">
+        <v>17</v>
+      </c>
+      <c r="D23" s="32">
+        <v>45959.104166666672</v>
+      </c>
+      <c r="E23" s="32">
+        <v>45959.104166666672</v>
+      </c>
+      <c r="F23" s="30">
+        <v>59</v>
+      </c>
+      <c r="G23" s="33">
+        <f>ROUND(14.71*25.4,1)</f>
+        <v>373.6</v>
+      </c>
+      <c r="H23" s="30"/>
+      <c r="I23" s="31" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="112" x14ac:dyDescent="0.2">
+      <c r="A24" s="30">
+        <v>18</v>
+      </c>
+      <c r="B24" s="30">
+        <v>0</v>
+      </c>
+      <c r="C24" s="30">
+        <v>18</v>
+      </c>
+      <c r="D24" s="32">
+        <v>45959.076388888883</v>
+      </c>
+      <c r="E24" s="32">
+        <v>45959.076388888883</v>
+      </c>
+      <c r="F24" s="30">
+        <v>70</v>
+      </c>
+      <c r="G24" s="33">
+        <f>ROUND(13.2*25.4,1)</f>
+        <v>335.3</v>
+      </c>
+      <c r="H24" s="30"/>
+      <c r="I24" s="31" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="112" x14ac:dyDescent="0.2">
+      <c r="A25" s="30">
+        <v>19</v>
+      </c>
+      <c r="B25" s="30">
+        <v>0</v>
+      </c>
+      <c r="C25" s="30">
+        <v>19</v>
+      </c>
+      <c r="D25" s="32">
+        <v>45959.32708333333</v>
+      </c>
+      <c r="E25" s="32">
+        <v>45959.32708333333</v>
+      </c>
+      <c r="F25" s="30">
+        <v>51</v>
+      </c>
+      <c r="G25" s="33">
+        <f>ROUND(6.5*25.4,1)</f>
+        <v>165.1</v>
+      </c>
+      <c r="H25" s="30"/>
+      <c r="I25" s="31" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="96" x14ac:dyDescent="0.2">
+      <c r="A26" s="30">
+        <v>20</v>
+      </c>
+      <c r="B26" s="30">
+        <v>0</v>
+      </c>
+      <c r="C26" s="30">
+        <v>20</v>
+      </c>
+      <c r="D26" s="32">
+        <v>45959.489583333336</v>
+      </c>
+      <c r="E26" s="32">
+        <v>45959.489583333336</v>
+      </c>
+      <c r="F26" s="30">
+        <v>62</v>
+      </c>
+      <c r="G26" s="33">
+        <f>ROUND(10.84*25.4,1)</f>
+        <v>275.3</v>
+      </c>
+      <c r="H26" s="30"/>
+      <c r="I26" s="31" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="96" x14ac:dyDescent="0.2">
+      <c r="A27" s="30">
+        <v>21</v>
+      </c>
+      <c r="B27" s="30">
+        <v>0</v>
+      </c>
+      <c r="C27" s="30">
+        <v>21</v>
+      </c>
+      <c r="D27" s="32">
+        <v>45959.083333333336</v>
+      </c>
+      <c r="E27" s="32">
+        <v>45959.083333333336</v>
+      </c>
+      <c r="F27" s="30">
+        <v>47</v>
+      </c>
+      <c r="G27" s="33">
+        <f>ROUND(4.04*25.4,1)</f>
+        <v>102.6</v>
+      </c>
+      <c r="H27" s="30"/>
+      <c r="I27" s="31" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="96" x14ac:dyDescent="0.2">
+      <c r="A28" s="30">
+        <v>22</v>
+      </c>
+      <c r="B28" s="30">
+        <v>0</v>
+      </c>
+      <c r="C28" s="30">
+        <v>22</v>
+      </c>
+      <c r="D28" s="32">
+        <v>45959.853472222225</v>
+      </c>
+      <c r="E28" s="32">
+        <v>45959.853472222225</v>
+      </c>
+      <c r="F28" s="30">
+        <v>66</v>
+      </c>
+      <c r="G28" s="33"/>
+      <c r="H28" s="30"/>
+      <c r="I28" s="31" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="80" x14ac:dyDescent="0.2">
+      <c r="A29" s="30">
+        <v>23</v>
+      </c>
+      <c r="B29" s="30">
+        <v>0</v>
+      </c>
+      <c r="C29" s="30">
+        <v>23</v>
+      </c>
+      <c r="D29" s="32">
+        <v>45960.006249999999</v>
+      </c>
+      <c r="E29" s="32">
+        <v>45960.006249999999</v>
+      </c>
+      <c r="F29" s="30">
+        <v>45</v>
+      </c>
+      <c r="G29" s="33"/>
+      <c r="H29" s="30"/>
+      <c r="I29" s="31" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="96" x14ac:dyDescent="0.2">
+      <c r="A30" s="30">
+        <v>24</v>
+      </c>
+      <c r="B30" s="30">
+        <v>0</v>
+      </c>
+      <c r="C30" s="30">
+        <v>24</v>
+      </c>
+      <c r="D30" s="32">
+        <v>45959.870833333334</v>
+      </c>
+      <c r="E30" s="32">
+        <v>45959.870833333334</v>
+      </c>
+      <c r="F30" s="30">
+        <v>35</v>
+      </c>
+      <c r="G30" s="33"/>
+      <c r="H30" s="30"/>
+      <c r="I30" s="31" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" ht="64" x14ac:dyDescent="0.2">
+      <c r="A31" s="30">
+        <v>25</v>
+      </c>
+      <c r="B31" s="30">
+        <v>0</v>
+      </c>
+      <c r="C31" s="30">
+        <v>25</v>
+      </c>
+      <c r="D31" s="32"/>
+      <c r="E31" s="32"/>
+      <c r="F31" s="30"/>
+      <c r="G31" s="33">
+        <v>198</v>
+      </c>
+      <c r="H31" s="30"/>
+      <c r="I31" s="31" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" ht="96" x14ac:dyDescent="0.2">
+      <c r="A32" s="30">
+        <v>26</v>
+      </c>
+      <c r="B32" s="30">
+        <v>0</v>
+      </c>
+      <c r="C32" s="30">
+        <v>26</v>
+      </c>
+      <c r="D32" s="32">
+        <v>45961.163194444445</v>
+      </c>
+      <c r="E32" s="32">
+        <v>45961.163194444445</v>
+      </c>
+      <c r="F32" s="30">
+        <v>43</v>
+      </c>
+      <c r="G32" s="33"/>
+      <c r="H32" s="30"/>
+      <c r="I32" s="31" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="96" x14ac:dyDescent="0.2">
+      <c r="A33" s="30">
+        <v>27</v>
+      </c>
+      <c r="B33" s="30">
+        <v>0</v>
+      </c>
+      <c r="C33" s="30">
+        <v>27</v>
+      </c>
+      <c r="D33" s="32">
+        <v>45961.15625</v>
+      </c>
+      <c r="E33" s="32">
+        <v>45961.15625</v>
+      </c>
+      <c r="F33" s="30">
+        <v>68</v>
+      </c>
+      <c r="G33" s="33"/>
+      <c r="H33" s="30"/>
+      <c r="I33" s="31" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="80" x14ac:dyDescent="0.2">
+      <c r="A34" s="30">
+        <v>28</v>
+      </c>
+      <c r="B34" s="30">
+        <v>0</v>
+      </c>
+      <c r="C34" s="30">
+        <v>28</v>
+      </c>
+      <c r="D34" s="32"/>
+      <c r="E34" s="32"/>
+      <c r="F34" s="30"/>
+      <c r="G34" s="33">
+        <v>893</v>
+      </c>
+      <c r="H34" s="30"/>
+      <c r="I34" s="31" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="64" x14ac:dyDescent="0.2">
+      <c r="A35" s="30">
+        <v>29</v>
+      </c>
+      <c r="B35" s="30">
+        <v>0</v>
+      </c>
+      <c r="C35" s="30">
+        <v>29</v>
+      </c>
+      <c r="D35" s="32"/>
+      <c r="E35" s="32"/>
+      <c r="F35" s="30"/>
+      <c r="G35" s="33">
+        <v>856.5</v>
+      </c>
+      <c r="H35" s="30"/>
+      <c r="I35" s="31" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="64" x14ac:dyDescent="0.2">
+      <c r="A36" s="30">
+        <v>30</v>
+      </c>
+      <c r="B36" s="30">
+        <v>0</v>
+      </c>
+      <c r="C36" s="30">
+        <v>30</v>
+      </c>
+      <c r="D36" s="32"/>
+      <c r="E36" s="32"/>
+      <c r="F36" s="30"/>
+      <c r="G36" s="33">
+        <v>835.6</v>
+      </c>
+      <c r="H36" s="30"/>
+      <c r="I36" s="31" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="64" x14ac:dyDescent="0.2">
+      <c r="A37" s="30">
+        <v>31</v>
+      </c>
+      <c r="B37" s="30">
+        <v>0</v>
+      </c>
+      <c r="C37" s="30">
+        <v>31</v>
+      </c>
+      <c r="D37" s="32"/>
+      <c r="E37" s="32"/>
+      <c r="F37" s="30"/>
+      <c r="G37" s="33">
+        <v>737.2</v>
+      </c>
+      <c r="H37" s="30"/>
+      <c r="I37" s="31" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="64" x14ac:dyDescent="0.2">
+      <c r="A38" s="30">
+        <v>32</v>
+      </c>
+      <c r="B38" s="30">
+        <v>0</v>
+      </c>
+      <c r="C38" s="30">
+        <v>32</v>
+      </c>
+      <c r="D38" s="32"/>
+      <c r="E38" s="32"/>
+      <c r="F38" s="30"/>
+      <c r="G38" s="33">
+        <v>507.4</v>
+      </c>
+      <c r="H38" s="30"/>
+      <c r="I38" s="31" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="64" x14ac:dyDescent="0.2">
+      <c r="A39" s="30">
+        <v>33</v>
+      </c>
+      <c r="B39" s="30">
+        <v>0</v>
+      </c>
+      <c r="C39" s="30">
+        <v>33</v>
+      </c>
+      <c r="D39" s="32"/>
+      <c r="E39" s="32"/>
+      <c r="F39" s="30"/>
+      <c r="G39" s="33">
+        <v>453.1</v>
+      </c>
+      <c r="H39" s="30"/>
+      <c r="I39" s="31" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="80" x14ac:dyDescent="0.2">
+      <c r="A40" s="30">
+        <v>34</v>
+      </c>
+      <c r="B40" s="30">
+        <v>0</v>
+      </c>
+      <c r="C40" s="30">
+        <v>34</v>
+      </c>
+      <c r="D40" s="32"/>
+      <c r="E40" s="32"/>
+      <c r="F40" s="30"/>
+      <c r="G40" s="33"/>
+      <c r="H40" s="30"/>
+      <c r="I40" s="31" t="s">
+        <v>201</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
@@ -6545,7 +7638,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3528AC7-2802-4014-B630-EA5F377DA589}">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
@@ -6671,8 +7764,58 @@
         <v>105</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="G9" s="27"/>
+    <row r="9" spans="1:7" ht="64" x14ac:dyDescent="0.2">
+      <c r="A9" s="30">
+        <v>3</v>
+      </c>
+      <c r="B9" s="30">
+        <v>34</v>
+      </c>
+      <c r="C9" s="30"/>
+      <c r="D9" s="30"/>
+      <c r="E9" s="34"/>
+      <c r="F9" s="34"/>
+      <c r="G9" s="31" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="64" x14ac:dyDescent="0.2">
+      <c r="A10" s="30">
+        <v>4</v>
+      </c>
+      <c r="B10" s="30">
+        <v>26</v>
+      </c>
+      <c r="C10" s="30">
+        <v>0</v>
+      </c>
+      <c r="D10" s="30">
+        <v>0</v>
+      </c>
+      <c r="E10" s="34"/>
+      <c r="F10" s="34"/>
+      <c r="G10" s="31" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="80" x14ac:dyDescent="0.2">
+      <c r="A11" s="30">
+        <v>5</v>
+      </c>
+      <c r="B11" s="30">
+        <v>31</v>
+      </c>
+      <c r="C11" s="30">
+        <v>0</v>
+      </c>
+      <c r="D11" s="30">
+        <v>0</v>
+      </c>
+      <c r="E11" s="34"/>
+      <c r="F11" s="34"/>
+      <c r="G11" s="31" t="s">
+        <v>204</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -6686,7 +7829,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F10B1DA-B875-4400-86A1-B83B41030127}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.5" customWidth="1"/>
@@ -6828,6 +7971,578 @@
       <c r="E9" s="23"/>
       <c r="F9" s="24" t="s">
         <v>97</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+      <c r="A10" s="30">
+        <v>4</v>
+      </c>
+      <c r="B10" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="C10" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="D10" s="30">
+        <v>18.09</v>
+      </c>
+      <c r="E10" s="30">
+        <v>-77.97</v>
+      </c>
+      <c r="F10" s="31" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+      <c r="A11" s="30">
+        <v>5</v>
+      </c>
+      <c r="B11" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="C11" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="D11" s="30">
+        <v>18.440000000000001</v>
+      </c>
+      <c r="E11" s="30">
+        <v>-77.75</v>
+      </c>
+      <c r="F11" s="31" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+      <c r="A12" s="30">
+        <v>6</v>
+      </c>
+      <c r="B12" s="30" t="s">
+        <v>110</v>
+      </c>
+      <c r="C12" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="D12" s="30">
+        <v>18.399999999999999</v>
+      </c>
+      <c r="E12" s="30">
+        <v>-77.28</v>
+      </c>
+      <c r="F12" s="31" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+      <c r="A13" s="30">
+        <v>7</v>
+      </c>
+      <c r="B13" s="30" t="s">
+        <v>112</v>
+      </c>
+      <c r="C13" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="D13" s="30">
+        <v>18.170000000000002</v>
+      </c>
+      <c r="E13" s="30">
+        <v>-77.72</v>
+      </c>
+      <c r="F13" s="31" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+      <c r="A14" s="30">
+        <v>8</v>
+      </c>
+      <c r="B14" s="30" t="s">
+        <v>114</v>
+      </c>
+      <c r="C14" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="D14" s="30">
+        <v>17.98</v>
+      </c>
+      <c r="E14" s="30">
+        <v>-77.75</v>
+      </c>
+      <c r="F14" s="31" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+      <c r="A15" s="30">
+        <v>9</v>
+      </c>
+      <c r="B15" s="30" t="s">
+        <v>116</v>
+      </c>
+      <c r="C15" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="D15" s="30">
+        <v>17.920000000000002</v>
+      </c>
+      <c r="E15" s="30">
+        <v>-77.760000000000005</v>
+      </c>
+      <c r="F15" s="31" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+      <c r="A16" s="30">
+        <v>10</v>
+      </c>
+      <c r="B16" s="30" t="s">
+        <v>118</v>
+      </c>
+      <c r="C16" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="D16" s="30">
+        <v>18.47</v>
+      </c>
+      <c r="E16" s="30">
+        <v>-77.73</v>
+      </c>
+      <c r="F16" s="31" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+      <c r="A17" s="30">
+        <v>11</v>
+      </c>
+      <c r="B17" s="30" t="s">
+        <v>120</v>
+      </c>
+      <c r="C17" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="D17" s="30">
+        <v>18.41</v>
+      </c>
+      <c r="E17" s="30">
+        <v>-77.38</v>
+      </c>
+      <c r="F17" s="31" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+      <c r="A18" s="30">
+        <v>12</v>
+      </c>
+      <c r="B18" s="30" t="s">
+        <v>122</v>
+      </c>
+      <c r="C18" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="D18" s="30">
+        <v>18.2</v>
+      </c>
+      <c r="E18" s="30">
+        <v>-77.260000000000005</v>
+      </c>
+      <c r="F18" s="31" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+      <c r="A19" s="30">
+        <v>13</v>
+      </c>
+      <c r="B19" s="30" t="s">
+        <v>124</v>
+      </c>
+      <c r="C19" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="D19" s="30">
+        <v>18.07</v>
+      </c>
+      <c r="E19" s="30">
+        <v>-76.75</v>
+      </c>
+      <c r="F19" s="31" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+      <c r="A20" s="30">
+        <v>14</v>
+      </c>
+      <c r="B20" s="30" t="s">
+        <v>126</v>
+      </c>
+      <c r="C20" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="D20" s="30">
+        <v>18.03</v>
+      </c>
+      <c r="E20" s="30">
+        <v>-76.650000000000006</v>
+      </c>
+      <c r="F20" s="31" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+      <c r="A21" s="30">
+        <v>15</v>
+      </c>
+      <c r="B21" s="30" t="s">
+        <v>128</v>
+      </c>
+      <c r="C21" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="D21" s="30">
+        <v>18.5</v>
+      </c>
+      <c r="E21" s="30">
+        <v>-77.91</v>
+      </c>
+      <c r="F21" s="31" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+      <c r="A22" s="30">
+        <v>16</v>
+      </c>
+      <c r="B22" s="30" t="s">
+        <v>130</v>
+      </c>
+      <c r="C22" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="D22" s="30">
+        <v>17.940000000000001</v>
+      </c>
+      <c r="E22" s="30">
+        <v>-76.77</v>
+      </c>
+      <c r="F22" s="31" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+      <c r="A23" s="30">
+        <v>17</v>
+      </c>
+      <c r="B23" s="30" t="s">
+        <v>132</v>
+      </c>
+      <c r="C23" s="30" t="s">
+        <v>90</v>
+      </c>
+      <c r="D23" s="30"/>
+      <c r="E23" s="30"/>
+      <c r="F23" s="31" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+      <c r="A24" s="30">
+        <v>18</v>
+      </c>
+      <c r="B24" s="30" t="s">
+        <v>134</v>
+      </c>
+      <c r="C24" s="30" t="s">
+        <v>90</v>
+      </c>
+      <c r="D24" s="30"/>
+      <c r="E24" s="30"/>
+      <c r="F24" s="31" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+      <c r="A25" s="30">
+        <v>19</v>
+      </c>
+      <c r="B25" s="30" t="s">
+        <v>136</v>
+      </c>
+      <c r="C25" s="30" t="s">
+        <v>90</v>
+      </c>
+      <c r="D25" s="30"/>
+      <c r="E25" s="30"/>
+      <c r="F25" s="31" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+      <c r="A26" s="30">
+        <v>20</v>
+      </c>
+      <c r="B26" s="30" t="s">
+        <v>138</v>
+      </c>
+      <c r="C26" s="30" t="s">
+        <v>90</v>
+      </c>
+      <c r="D26" s="30"/>
+      <c r="E26" s="30"/>
+      <c r="F26" s="31" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+      <c r="A27" s="30">
+        <v>21</v>
+      </c>
+      <c r="B27" s="30" t="s">
+        <v>140</v>
+      </c>
+      <c r="C27" s="30" t="s">
+        <v>90</v>
+      </c>
+      <c r="D27" s="30"/>
+      <c r="E27" s="30"/>
+      <c r="F27" s="31" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+      <c r="A28" s="30">
+        <v>22</v>
+      </c>
+      <c r="B28" s="30" t="s">
+        <v>142</v>
+      </c>
+      <c r="C28" s="30" t="s">
+        <v>93</v>
+      </c>
+      <c r="D28" s="30">
+        <v>22.83</v>
+      </c>
+      <c r="E28" s="30">
+        <v>-74.34</v>
+      </c>
+      <c r="F28" s="31" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+      <c r="A29" s="30">
+        <v>23</v>
+      </c>
+      <c r="B29" s="30" t="s">
+        <v>144</v>
+      </c>
+      <c r="C29" s="30" t="s">
+        <v>93</v>
+      </c>
+      <c r="D29" s="30">
+        <v>23.36</v>
+      </c>
+      <c r="E29" s="30">
+        <v>-75.150000000000006</v>
+      </c>
+      <c r="F29" s="31" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+      <c r="A30" s="30">
+        <v>24</v>
+      </c>
+      <c r="B30" s="30" t="s">
+        <v>146</v>
+      </c>
+      <c r="C30" s="30" t="s">
+        <v>93</v>
+      </c>
+      <c r="D30" s="30">
+        <v>23.16</v>
+      </c>
+      <c r="E30" s="30">
+        <v>-75.09</v>
+      </c>
+      <c r="F30" s="31" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+      <c r="A31" s="30">
+        <v>25</v>
+      </c>
+      <c r="B31" s="30" t="s">
+        <v>148</v>
+      </c>
+      <c r="C31" s="30" t="s">
+        <v>93</v>
+      </c>
+      <c r="D31" s="30">
+        <v>24.11</v>
+      </c>
+      <c r="E31" s="30">
+        <v>-74.45</v>
+      </c>
+      <c r="F31" s="31" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+      <c r="A32" s="30">
+        <v>26</v>
+      </c>
+      <c r="B32" s="30" t="s">
+        <v>150</v>
+      </c>
+      <c r="C32" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="D32" s="30">
+        <v>32.36</v>
+      </c>
+      <c r="E32" s="30">
+        <v>-64.680000000000007</v>
+      </c>
+      <c r="F32" s="31" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+      <c r="A33" s="30">
+        <v>27</v>
+      </c>
+      <c r="B33" s="30" t="s">
+        <v>153</v>
+      </c>
+      <c r="C33" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="D33" s="30">
+        <v>32.33</v>
+      </c>
+      <c r="E33" s="30">
+        <v>-64.83</v>
+      </c>
+      <c r="F33" s="31" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+      <c r="A34" s="30">
+        <v>28</v>
+      </c>
+      <c r="B34" s="30" t="s">
+        <v>155</v>
+      </c>
+      <c r="C34" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="D34" s="30"/>
+      <c r="E34" s="30"/>
+      <c r="F34" s="31" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+      <c r="A35" s="30">
+        <v>29</v>
+      </c>
+      <c r="B35" s="30" t="s">
+        <v>157</v>
+      </c>
+      <c r="C35" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="D35" s="30"/>
+      <c r="E35" s="30"/>
+      <c r="F35" s="31" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+      <c r="A36" s="30">
+        <v>30</v>
+      </c>
+      <c r="B36" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="C36" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="D36" s="30"/>
+      <c r="E36" s="30"/>
+      <c r="F36" s="31" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+      <c r="A37" s="30">
+        <v>31</v>
+      </c>
+      <c r="B37" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="C37" s="30" t="s">
+        <v>162</v>
+      </c>
+      <c r="D37" s="30"/>
+      <c r="E37" s="30"/>
+      <c r="F37" s="31" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+      <c r="A38" s="30">
+        <v>32</v>
+      </c>
+      <c r="B38" s="30" t="s">
+        <v>164</v>
+      </c>
+      <c r="C38" s="30" t="s">
+        <v>162</v>
+      </c>
+      <c r="D38" s="30"/>
+      <c r="E38" s="30"/>
+      <c r="F38" s="31" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+      <c r="A39" s="30">
+        <v>33</v>
+      </c>
+      <c r="B39" s="30" t="s">
+        <v>166</v>
+      </c>
+      <c r="C39" s="30" t="s">
+        <v>162</v>
+      </c>
+      <c r="D39" s="30"/>
+      <c r="E39" s="30"/>
+      <c r="F39" s="31" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+      <c r="A40" s="30">
+        <v>34</v>
+      </c>
+      <c r="B40" s="30" t="s">
+        <v>168</v>
+      </c>
+      <c r="C40" s="30" t="s">
+        <v>169</v>
+      </c>
+      <c r="D40" s="30"/>
+      <c r="E40" s="30"/>
+      <c r="F40" s="31" t="s">
+        <v>170</v>
       </c>
     </row>
   </sheetData>

</xml_diff>